<commit_message>
Add Odoo 19 sample files and set version 19.0.1.0.0
</commit_message>
<xml_diff>
--- a/sm_import_order_lines/sample_import_order_lines.xlsx
+++ b/sm_import_order_lines/sample_import_order_lines.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Product Code / Name</t>
+          <t>Product Code</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -429,7 +429,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Unit Price</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>E-COM12</t>
+          <t>FURN_2100</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -452,14 +452,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Black Leather Chair</t>
+          <t>Drawer Black</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>E-COM13</t>
+          <t>FURN_7777</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -470,43 +470,43 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>White Leather Chair</t>
+          <t>Office Chair</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CONS_0001</t>
+          <t>FURN_9666</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>2.5</v>
+        <v>250</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Blue Marker</t>
+          <t>Table Top Executive</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CONS_0002</t>
+          <t>CONS_0001</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Red Pen</t>
+          <t>Whiteboard Marker Pen Blue</t>
         </is>
       </c>
     </row>

</xml_diff>